<commit_message>
docs: remake Sinops-11/12/21 Phase1 packs and align 24/25 master integration
Refresh nyuka/uke mapping·GAP·rules from Seiyu IF layout upgrades, and pin store/supplier/product links to master unification on 24/25 DD.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/PMI/Sinops/phase2-detail-design/DD/Sinops-24_発注勧告当日_IF詳細設計書.xlsx
+++ b/PMI/Sinops/phase2-detail-design/DD/Sinops-24_発注勧告当日_IF詳細設計書.xlsx
@@ -1022,6 +1022,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1596,20 +1599,70 @@
       <c r="G24" s="23" t="n"/>
     </row>
     <row r="25" ht="21.75" customHeight="1">
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D25" s="25" t="inlineStr">
+        <is>
+          <t>臧鵬仕</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>Ordertype：部門CDは勧告ファイルの西友中分類（西友ライン）。TRIAL商品マスタは参照しない</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="n"/>
+      <c r="G25" s="23" t="n"/>
     </row>
     <row r="26" ht="21.75" customHeight="1">
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D26" s="25" t="inlineStr">
+        <is>
+          <t>臧鵬仕</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>店CD・商品の紐付けは西友（Sinops）とTRIALのマスタ統合で解決。本IFは独自変換しない</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="n"/>
+      <c r="G26" s="23" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D27" s="25" t="inlineStr">
+        <is>
+          <t>臧鵬仕</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>仕入先マスタも統合作業。本IFは9→8の独自変換をしない</t>
+        </is>
+      </c>
+      <c r="F27" s="26" t="n"/>
+      <c r="G27" s="23" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="2" t="inlineStr">
@@ -1737,7 +1790,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>店舗コード6桁を BranchCD 4桁へどう変換するか。切捨て禁止</t>
+          <t>店舗コードとTRIAL店CDの紐付け。6桁→4桁の独自変換はしない</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -1757,10 +1810,14 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>確認中</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="inlineStr"/>
+          <t>一部確定</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>方針：西友（Sinops）とTRIALのマスタ統合により店舗の紐付けは解決する。本IFは独自の店CD変換・切捨てを持たない。出力桁は統合作業後のコード体系に従う</t>
+        </is>
+      </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
           <t>G-05 / G02</t>
@@ -2038,7 +2095,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>仕入先9桁→ベンダーCD 8桁。切捨て禁止</t>
+          <t>仕入先とTRIALベンダーの紐付け。9桁→8桁の独自変換はしない</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -2058,10 +2115,14 @@
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>確認中</t>
-        </is>
-      </c>
-      <c r="I13" s="10" t="inlineStr"/>
+          <t>一部確定</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>方針：仕入先マスタもマスタ統合で紐付けが解決する。本IFは独自のベンダーCD切捨て・変換を持たない。出力は統合作業後のコード体系に従う</t>
+        </is>
+      </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
           <t>G03</t>
@@ -2081,7 +2142,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Ordertype 1桁の値定義。sinopsに項目なし</t>
+          <t>Ordertype 1桁の値定義。sinopsにOrdertype項目なし。部門は勧告ファイルにある</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -2106,7 +2167,7 @@
       </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
-          <t>0=非日配、1=日配または生鮮。TRIAL商品マスタ部門階層の部門CD → 自動発注GCS JIHA.BUMON_ZONE → JIHA.ZONE_LOGIC。論理区分 01→0、02→1、03→1</t>
+          <t>0=非日配、1=日配または生鮮。部門CDは勧告ファイルの西友中分類（西友ライン）。商品マスタは見ない。JIHA.BUMON_ZONE → JIHA.ZONE_LOGIC。01→0、02→1、03→1</t>
         </is>
       </c>
       <c r="J14" s="10" t="inlineStr">
@@ -2171,7 +2232,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>SireJAN が通常JANと同一か、仕入JAN変換が要るか</t>
+          <t>SireJANとTRIAL商品の紐付け。独自の仕入JAN変換はしない</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -2191,10 +2252,14 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>確認中</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="inlineStr"/>
+          <t>一部確定</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>方針：マスタ統合により商品の紐付けは解決する。本IFは独自の仕入JAN変換を持たない。SireJANは統合後の商品コードを載せる</t>
+        </is>
+      </c>
       <c r="J16" s="10" t="inlineStr">
         <is>
           <t>G11</t>
@@ -3451,12 +3516,12 @@
       </c>
       <c r="C17" s="51" t="inlineStr">
         <is>
-          <t>採用した 1 本を SIREJAN_RCMDORDER_LAST へ変換。数量は×1000しない。発注単位の整数倍であれば発注バラ数を直接設定（倍数に丸めない）。Ordertype は TRIAL 商品マスタの部門階層の部門CDで 自動発注GCS JIHA.BUMON_ZONE（部門CD, ZONECD）を引き、ZONECD で JIHA.ZONE_LOGIC（ZONECD, 論理区分）を結合。論理区分 01→0（非日配）、02→1（日配）、03→1（生鮮）</t>
+          <t>採用した 1 本を SIREJAN_RCMDORDER_LAST へ変換。数量は×1000しない。発注単位の整数倍であれば発注バラ数を直接設定（倍数に丸めない）。Ordertype は勧告ファイルの西友中分類（西友ライン＝部門）を部門CDとし、自動発注GCS JIHA.BUMON_ZONE（部門CD, ZONECD）→ JIHA.ZONE_LOGIC（ZONECD, 論理区分）。論理区分 01→0（非日配）、02→1（日配）、03→1（生鮮）。TRIAL 商品マスタは参照しない。</t>
         </is>
       </c>
       <c r="D17" s="50" t="inlineStr">
         <is>
-          <t>採用した 1 本 ＋ TRIAL商品マスタ部門 ＋ JIHA.BUMON_ZONE / JIHA.ZONE_LOGIC（自動発注GCS）</t>
+          <t>採用した 1 本（部門＝西友中分類／西友ライン）＋ JIHA.BUMON_ZONE / JIHA.ZONE_LOGIC（自動発注GCS）</t>
         </is>
       </c>
       <c r="E17" s="50" t="inlineStr">
@@ -3471,7 +3536,7 @@
       </c>
       <c r="G17" s="49" t="inlineStr">
         <is>
-          <t>R01/R04/R06/R07 確定。数量は発注単位の整数倍（×1000しない）。店CD・ベンダーは切捨て禁止</t>
+          <t>R01/R04/R06/R07 確定。部門は勧告ファイル。商品マスタは見ない。数量は発注単位の整数倍。店・仕入先・商品はマスタ統合に追随</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -4469,7 +4534,7 @@
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>R02／6桁→4桁は切捨て禁止。変換式 TBD-01</t>
+          <t>店CDの紐付けは西友（Sinops）とTRIALのマスタ統合で解決。本IFは6→4切捨て等の独自変換をしない。桁は統合作業に追随 TBD-01</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
@@ -4484,12 +4549,12 @@
       </c>
       <c r="S6" s="9" t="inlineStr">
         <is>
-          <t>未確定</t>
+          <t>一部確定</t>
         </is>
       </c>
       <c r="T6" s="9" t="inlineStr">
         <is>
-          <t>WBS Layer①</t>
+          <t>マスタ統合で紐付け解決</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4625,7 @@
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>R03／文字列・先頭ゼロ保持。仕入JAN定義 TBD-11</t>
+          <t>商品の紐付けはマスタ統合で解決。本IFは独自の仕入JAN変換をしない。SireJANは統合後の商品コード。先頭ゼロ保持</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
@@ -4578,7 +4643,11 @@
           <t>一部確定</t>
         </is>
       </c>
-      <c r="T7" s="9" t="inlineStr"/>
+      <c r="T7" s="9" t="inlineStr">
+        <is>
+          <t>マスタ統合で紐付け解決</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
       <c r="B8" s="8" t="n">
@@ -4730,7 +4799,7 @@
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>R05／9桁→8桁は切捨て禁止。変換式 TBD-08</t>
+          <t>仕入先マスタも西友（Sinops）とTRIALで統合。本IFは9→8切捨て等の独自変換をしない。桁は統合作業に追随 TBD-08</t>
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr">
@@ -4745,10 +4814,14 @@
       </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>未確定</t>
-        </is>
-      </c>
-      <c r="T9" s="10" t="inlineStr"/>
+          <t>一部確定</t>
+        </is>
+      </c>
+      <c r="T9" s="10" t="inlineStr">
+        <is>
+          <t>マスタ統合で紐付け解決</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
       <c r="B10" s="10" t="n">
@@ -4865,12 +4938,12 @@
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>TRIAL 商品マスタ（部門階層）／自動発注GCS JIHA.BUMON_ZONE／JIHA.ZONE_LOGIC</t>
+          <t>Sinops 勧告ファイル 西友中分類（西友ライン＝部門）／自動発注GCS JIHA.BUMON_ZONE／JIHA.ZONE_LOGIC</t>
         </is>
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>部門CD → ZONECD → 論理区分</t>
+          <t>部門（西友ライン）→ ZONECD → 論理区分</t>
         </is>
       </c>
       <c r="K11" s="10" t="inlineStr">
@@ -4900,7 +4973,7 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>R07／sinops項目なし。論理区分01→Ordertype=0（非日配）、02→1（日配）、03→1（生鮮）。参照：自動発注GCS JIHA.BUMON_ZONE（部門CD,ZONECD）、JIHA.ZONE_LOGIC（ZONECD,論理区分）。</t>
+          <t>R07／Ordertypeはsinopsに無い。部門CDは勧告ファイルの西友中分類（西友ライン＝階層4）。大分類（デパ）＝ディビジョン、小分類（ファインライン）＝カテゴリ、JAN＝単品JAN。TRIAL商品マスタは見ない。論理区分01→0、02→1、03→1。JIHA.BUMON_ZONE / ZONE_LOGIC（自動発注GCS）</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
@@ -4920,7 +4993,7 @@
       </c>
       <c r="T11" s="10" t="inlineStr">
         <is>
-          <t>Layer① で付与。Layer③ では作らない。02と03はどちらも1</t>
+          <t>Layer① で付与。商品マスタは見ない。02と03はどちらも1</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6235,7 @@
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>切捨て禁止 TBD-01</t>
+          <t>マスタ統合後の店CD。独自切捨てなし TBD-01</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr">
@@ -6210,7 +6283,7 @@
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>文字列・左ゼロ保持</t>
+          <t>マスタ統合後の商品コード。先頭ゼロ保持</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr"/>
@@ -6300,7 +6373,7 @@
       </c>
       <c r="J21" s="10" t="inlineStr">
         <is>
-          <t>切捨て禁止 TBD-08</t>
+          <t>マスタ統合後の仕入先CD。独自切捨てなし TBD-08</t>
         </is>
       </c>
       <c r="K21" s="10" t="inlineStr"/>
@@ -6384,7 +6457,7 @@
       </c>
       <c r="J23" s="10" t="inlineStr">
         <is>
-          <t>R07。論理区分01→0、02/03→1</t>
+          <t>R07。部門は勧告の西友ライン。商品マスタ見ない。01→0、02/03→1</t>
         </is>
       </c>
       <c r="K23" s="10" t="inlineStr">
@@ -8053,7 +8126,7 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>必須欠落、店CD/ベンダー切捨て発生、数量非数値、発注単位の整数倍でない（×1000しない・倍数に丸めない）</t>
+          <t>必須欠落、店CD・仕入先・商品が統合マスタと不一致、数量非数値、発注単位の整数倍でない（×1000しない・倍数に丸めない）</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -8197,7 +8270,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>部門CDが BUMON_ZONE に無い、または ZONE_LOGIC が引けない、または論理区分が 01/02/03 以外</t>
+          <t>勧告ファイルの部門（西友ライン）が BUMON_ZONE に無い、または ZONE_LOGIC が引けない、または論理区分が 01/02/03 以外</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">

</xml_diff>